<commit_message>
push otochem output file
</commit_message>
<xml_diff>
--- a/outputs/R_OUT - Otolith microchemstry results with biodata.xlsx
+++ b/outputs/R_OUT - Otolith microchemstry results with biodata.xlsx
@@ -11854,7 +11854,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -12168,7 +12168,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -12200,7 +12200,7 @@
       </c>
       <c r="AQ81" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR81" t="inlineStr">
@@ -12220,12 +12220,12 @@
       </c>
       <c r="AU81" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV81" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW81" t="inlineStr">
@@ -12320,7 +12320,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -12477,7 +12477,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -12634,7 +12634,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -12666,7 +12666,7 @@
       </c>
       <c r="AQ84" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR84" t="inlineStr">
@@ -12686,12 +12686,12 @@
       </c>
       <c r="AU84" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV84" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW84" t="inlineStr">
@@ -12781,7 +12781,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -12813,7 +12813,7 @@
       </c>
       <c r="AQ85" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR85" t="inlineStr">
@@ -12833,12 +12833,12 @@
       </c>
       <c r="AU85" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV85" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW85" t="inlineStr">
@@ -12928,7 +12928,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="AQ87" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR87" t="inlineStr">
@@ -13137,12 +13137,12 @@
       </c>
       <c r="AU87" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV87" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW87" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -13384,7 +13384,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -13416,7 +13416,7 @@
       </c>
       <c r="AQ89" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR89" t="inlineStr">
@@ -13436,12 +13436,12 @@
       </c>
       <c r="AU89" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV89" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW89" t="inlineStr">
@@ -13531,7 +13531,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr">
@@ -13563,7 +13563,7 @@
       </c>
       <c r="AQ90" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR90" t="inlineStr">
@@ -13583,12 +13583,12 @@
       </c>
       <c r="AU90" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV90" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW90" t="inlineStr">
@@ -13678,7 +13678,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -13835,7 +13835,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -13992,7 +13992,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -14149,7 +14149,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -14301,7 +14301,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -14333,7 +14333,7 @@
       </c>
       <c r="AQ95" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR95" t="inlineStr">
@@ -14353,12 +14353,12 @@
       </c>
       <c r="AU95" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV95" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW95" t="inlineStr">
@@ -14448,7 +14448,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="AQ96" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR96" t="inlineStr">
@@ -14500,12 +14500,12 @@
       </c>
       <c r="AU96" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV96" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW96" t="inlineStr">
@@ -14595,7 +14595,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -14627,7 +14627,7 @@
       </c>
       <c r="AQ97" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR97" t="inlineStr">
@@ -14647,12 +14647,12 @@
       </c>
       <c r="AU97" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV97" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW97" t="inlineStr">
@@ -14742,7 +14742,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="AQ98" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR98" t="inlineStr">
@@ -14794,12 +14794,12 @@
       </c>
       <c r="AU98" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV98" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW98" t="inlineStr">
@@ -14889,7 +14889,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="AQ99" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR99" t="inlineStr">
@@ -14941,12 +14941,12 @@
       </c>
       <c r="AU99" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV99" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW99" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -15188,7 +15188,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -15340,7 +15340,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -15372,7 +15372,7 @@
       </c>
       <c r="AQ102" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR102" t="inlineStr">
@@ -15392,12 +15392,12 @@
       </c>
       <c r="AU102" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV102" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW102" t="inlineStr">
@@ -15492,7 +15492,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -15644,7 +15644,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y104" t="inlineStr">
@@ -15676,7 +15676,7 @@
       </c>
       <c r="AQ104" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR104" t="inlineStr">
@@ -15696,12 +15696,12 @@
       </c>
       <c r="AU104" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV104" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW104" t="inlineStr">
@@ -15796,7 +15796,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y105" t="inlineStr">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y106" t="inlineStr">
@@ -15980,7 +15980,7 @@
       </c>
       <c r="AQ106" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR106" t="inlineStr">
@@ -16000,12 +16000,12 @@
       </c>
       <c r="AU106" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV106" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW106" t="inlineStr">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y107" t="inlineStr">
@@ -16252,7 +16252,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y108" t="inlineStr">
@@ -16284,7 +16284,7 @@
       </c>
       <c r="AQ108" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR108" t="inlineStr">
@@ -16304,12 +16304,12 @@
       </c>
       <c r="AU108" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV108" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW108" t="inlineStr">
@@ -16399,7 +16399,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y109" t="inlineStr">
@@ -16551,7 +16551,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y110" t="inlineStr">
@@ -16703,7 +16703,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y111" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="AQ111" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR111" t="inlineStr">
@@ -16755,12 +16755,12 @@
       </c>
       <c r="AU111" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV111" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW111" t="inlineStr">
@@ -16850,7 +16850,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y112" t="inlineStr">
@@ -17002,7 +17002,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y113" t="inlineStr">
@@ -17034,7 +17034,7 @@
       </c>
       <c r="AQ113" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR113" t="inlineStr">
@@ -17054,12 +17054,12 @@
       </c>
       <c r="AU113" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AV113" t="inlineStr">
         <is>
-          <t>Natural (assumed) San Juan River</t>
+          <t>Natural San Juan River</t>
         </is>
       </c>
       <c r="AW113" t="inlineStr">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y114" t="inlineStr">
@@ -17306,7 +17306,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y115" t="inlineStr">
@@ -17532,7 +17532,12 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>assume Chinook</t>
         </is>
       </c>
       <c r="AG117" t="inlineStr">
@@ -17542,28 +17547,51 @@
       </c>
       <c r="AQ117" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Hatchery</t>
+        </is>
+      </c>
+      <c r="AR117" t="inlineStr">
+        <is>
+          <t>PBT (presence/absence)</t>
         </is>
       </c>
       <c r="AS117" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>San Juan River</t>
+        </is>
+      </c>
+      <c r="AT117" t="inlineStr">
+        <is>
+          <t>PBT</t>
         </is>
       </c>
       <c r="AU117" t="inlineStr">
         <is>
-          <t>Unknown Unknown</t>
+          <t>Hatchery San Juan River</t>
         </is>
       </c>
       <c r="AV117" t="inlineStr">
         <is>
-          <t>Unknown Unknown</t>
+          <t>Hatchery San Juan River</t>
         </is>
       </c>
       <c r="AW117" t="inlineStr">
         <is>
-          <t>stray</t>
-        </is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="AX117" t="inlineStr">
+        <is>
+          <t>SAN_JUAN_RIVER</t>
+        </is>
+      </c>
+      <c r="AY117" t="inlineStr">
+        <is>
+          <t>SAN_JUAN_RIVER</t>
+        </is>
+      </c>
+      <c r="AZ117">
+        <v>100</v>
       </c>
     </row>
     <row r="118">
@@ -17634,7 +17662,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y118" t="inlineStr">
@@ -17666,7 +17694,7 @@
       </c>
       <c r="AQ118" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR118" t="inlineStr">
@@ -17681,17 +17709,17 @@
       </c>
       <c r="AU118" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AV118" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AW118" t="inlineStr">
         <is>
-          <t>stray</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="AY118" t="inlineStr">
@@ -17771,7 +17799,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y119" t="inlineStr">
@@ -17803,7 +17831,7 @@
       </c>
       <c r="AQ119" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR119" t="inlineStr">
@@ -17818,17 +17846,17 @@
       </c>
       <c r="AU119" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AV119" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AW119" t="inlineStr">
         <is>
-          <t>stray</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="AY119" t="inlineStr">
@@ -17908,7 +17936,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y120" t="inlineStr">
@@ -17940,7 +17968,7 @@
       </c>
       <c r="AQ120" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR120" t="inlineStr">
@@ -17960,12 +17988,12 @@
       </c>
       <c r="AU120" t="inlineStr">
         <is>
-          <t>Natural (assumed) Sooke River</t>
+          <t>Natural Sooke River</t>
         </is>
       </c>
       <c r="AV120" t="inlineStr">
         <is>
-          <t>Natural (assumed) Sooke/Nitinat</t>
+          <t>Natural Sooke/Nitinat</t>
         </is>
       </c>
       <c r="AW120" t="inlineStr">
@@ -18050,7 +18078,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y121" t="inlineStr">
@@ -18082,7 +18110,7 @@
       </c>
       <c r="AQ121" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR121" t="inlineStr">
@@ -18097,17 +18125,17 @@
       </c>
       <c r="AU121" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AV121" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AW121" t="inlineStr">
         <is>
-          <t>stray</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="AY121" t="inlineStr">
@@ -18187,7 +18215,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y122" t="inlineStr">
@@ -18219,7 +18247,7 @@
       </c>
       <c r="AQ122" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR122" t="inlineStr">
@@ -18239,12 +18267,12 @@
       </c>
       <c r="AU122" t="inlineStr">
         <is>
-          <t>Natural (assumed) Robertson Creek</t>
+          <t>Natural Robertson Creek</t>
         </is>
       </c>
       <c r="AV122" t="inlineStr">
         <is>
-          <t>Natural (assumed) Inner Barkley</t>
+          <t>Natural Inner Barkley</t>
         </is>
       </c>
       <c r="AW122" t="inlineStr">
@@ -18329,7 +18357,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y123" t="inlineStr">
@@ -18361,7 +18389,7 @@
       </c>
       <c r="AQ123" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR123" t="inlineStr">
@@ -18381,12 +18409,12 @@
       </c>
       <c r="AU123" t="inlineStr">
         <is>
-          <t>Natural (assumed) Sooke River</t>
+          <t>Natural Sooke River</t>
         </is>
       </c>
       <c r="AV123" t="inlineStr">
         <is>
-          <t>Natural (assumed) Sooke/Nitinat</t>
+          <t>Natural Sooke/Nitinat</t>
         </is>
       </c>
       <c r="AW123" t="inlineStr">
@@ -18471,7 +18499,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>Chinook</t>
         </is>
       </c>
       <c r="Y124" t="inlineStr">
@@ -18503,7 +18531,7 @@
       </c>
       <c r="AQ124" t="inlineStr">
         <is>
-          <t>Natural (assumed)</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="AR124" t="inlineStr">
@@ -18518,17 +18546,17 @@
       </c>
       <c r="AU124" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AV124" t="inlineStr">
         <is>
-          <t>Natural (assumed) Unknown</t>
+          <t>Natural Unknown</t>
         </is>
       </c>
       <c r="AW124" t="inlineStr">
         <is>
-          <t>stray</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="AY124" t="inlineStr">

</xml_diff>